<commit_message>
remove exteral excel dependencies and recalibrate emissions from luc
</commit_message>
<xml_diff>
--- a/Regionalized FeliX/Model Files/InitialValues.xlsx
+++ b/Regionalized FeliX/Model Files/InitialValues.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1240" documentId="13_ncr:1_{28C6C791-891C-49C6-B485-EBA1BBBF38AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{489CE2D8-5557-4E08-90DF-EBE422DB1238}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5856" yWindow="2124" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="936" yWindow="2100" windowWidth="17280" windowHeight="8880" tabRatio="623" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stocks" sheetId="1" r:id="rId1"/>

</xml_diff>